<commit_message>
Refine application features and supporting implementation
</commit_message>
<xml_diff>
--- a/DOCUMENT ESR/Capital décès Agent en activité.xlsx
+++ b/DOCUMENT ESR/Capital décès Agent en activité.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C802EBE3-F933-4827-B9BE-DED504119816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85064469-2046-4D5D-A942-0E80545AE9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HYPPOTHESE ACTUARIELLE" sheetId="4" r:id="rId1"/>
@@ -141,6 +141,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -532,9 +541,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -552,6 +558,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -633,6 +642,9 @@
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="TABLE DE MORTALITE"/>
       <sheetName val="Tarification"/>
@@ -692,6 +704,9 @@
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="DONNEES TECH"/>
       <sheetName val="Table SALARIE"/>
@@ -1395,6 +1410,9 @@
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="TABLE DE MORTALITE"/>
       <sheetName val="PRECOMPTE REVALORISER"/>
@@ -1702,24 +1720,24 @@
     <tabColor rgb="FFC00000"/>
   </sheetPr>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
     </row>
-    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1731,7 +1749,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="39.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="26.25" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1743,7 +1761,7 @@
         <v>8.6374459977134332E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="39" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
@@ -1755,7 +1773,7 @@
         <v>0.96618357487922713</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -1766,7 +1784,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -1777,7 +1795,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="7" t="s">
         <v>11</v>
       </c>
@@ -1788,7 +1806,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A9" s="10" t="s">
         <v>13</v>
       </c>
@@ -1797,10 +1815,10 @@
       </c>
       <c r="C9" s="11">
         <f ca="1">TODAY()</f>
-        <v>46226</v>
+        <v>46238</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:3" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C2"/>
@@ -1815,35 +1833,35 @@
     <tabColor theme="8" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="B2:N13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" style="1" customWidth="1"/>
-    <col min="3" max="4" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.86328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.3984375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="13.59765625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.265625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.73046875" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.42578125" style="1"/>
+    <col min="10" max="10" width="17.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.3984375" style="1"/>
     <col min="13" max="13" width="11" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.42578125" style="1"/>
+    <col min="14" max="16384" width="11.3984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:14" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C3" s="22" t="s">
+    <row r="2" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="3" spans="2:14" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="C3" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="23"/>
     </row>
-    <row r="4" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
@@ -1853,19 +1871,19 @@
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
     </row>
-    <row r="5" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:14" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="C5" s="13"/>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="27"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="26"/>
       <c r="H5" s="13"/>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
     </row>
-    <row r="8" spans="2:14" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" ht="60.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="15" t="s">
         <v>15</v>
       </c>
@@ -1897,7 +1915,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="2:14" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="17" t="s">
         <v>26</v>
       </c>
@@ -1930,17 +1948,17 @@
         <v>624952.00183137099</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.45">
       <c r="E11" s="12"/>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.45">
       <c r="H12" s="12">
         <v>0</v>
       </c>
       <c r="J12" s="12"/>
       <c r="M12" s="14"/>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.45">
       <c r="F13" s="12"/>
       <c r="N13" s="14"/>
     </row>

</xml_diff>